<commit_message>
docs(analyses): TP M3-1 — ligne 9 rattachee au cas A (chute)
Le support du module 3 indique que les equipes EHPAD relevent du cas A.
La justification reprend les trois lectures possibles de la promesse
(securite, prevention, prediction) et explique pourquoi la notre est
medicale.
</commit_message>
<xml_diff>
--- a/analyses/m3/grille_classification_eq05.xlsx
+++ b/analyses/m3/grille_classification_eq05.xlsx
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Projet 2 — Détection et prédiction de malaise et de chute en EHPAD, 20+ résidents (lettre du cas A à F à confirmer)</t>
+          <t>Cas A (chute) — Projet 2 : détection et prédiction de malaise et de chute en EHPAD, 20+ résidents</t>
         </is>
       </c>
       <c r="C13" s="10" t="n"/>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="J13" s="10" t="inlineStr">
         <is>
-          <t>Logiciel qui surveille des paramètres vitaux (fréquence cardiaque, SpO2, mouvement) dans une situation où un retard d'alerte met la vie en danger → règle 11, classe IIb ; IIa si l'on ne revendique qu'une surveillance sans urgence vitale. Dès IIa, organisme notifié obligatoire (GMED en France). (à vérifier)</t>
+          <t>Logiciel qui surveille des paramètres vitaux (fréquence cardiaque, SpO2, mouvement) dans une situation où un retard d'alerte peut être fatal → règle 11, classe IIb ; IIa si l'on ne revendiquait qu'une surveillance sans urgence vitale. Notre phrase va plus loin que « alerte quand un résident tombe » : elle promet de prédire le risque, donc de la prévention et de la prédiction — lecture médicale. Dès IIa, organisme notifié obligatoire (GMED en France). (à vérifier)</t>
         </is>
       </c>
       <c r="K13" s="11">

</xml_diff>